<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-08-31
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.503</v>
+        <v>3.456</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>101.66</v>
+        <v>10.5</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,48 +652,48 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>-1</v>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-9.640000000000001</v>
+        <v>10.49</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-1.77</v>
+        <v>2.95</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-0.52</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.671</v>
+        <v>1.496</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>99.95999999999999</v>
+        <v>101.66</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -711,44 +711,42 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-28.48</v>
+        <v>-9.01</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-10.94</v>
+        <v>-2.49</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>2.33</v>
+        <v>-1.24</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-1.49</v>
+        <v>-3.13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.551</v>
+        <v>0.666</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>101.36</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -758,11 +756,9 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -770,105 +766,113 @@
       <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>27.91</v>
+        <v>-28.09</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>10.7</v>
+        <v>-11.8</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-2.16</v>
+        <v>0.17</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>4.27</v>
+        <v>-2.43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.862</v>
+        <v>1.63</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>101.36</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-6.88</v>
+        <v>29.43</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.19</v>
+        <v>15.88</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-3.05</v>
+        <v>2.1</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>2.97</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.037</v>
+        <v>0.848</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44.27</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
@@ -877,43 +881,39 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.58</v>
+        <v>-6.08</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>0.88</v>
+        <v>-0.71</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>1.78</v>
+        <v>-1.22</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.15</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.679</v>
+        <v>3.041</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>21.63</v>
+        <v>44.27</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -930,41 +930,43 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-0.34</v>
+        <v>-2.55</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.29</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.16</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-0.05</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.923</v>
+        <v>4.685</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>17.83</v>
+        <v>21.63</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -976,7 +978,7 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
@@ -990,152 +992,148 @@
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>0.66</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>3.55</v>
+        <v>1.05</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.76</v>
+        <v>-0.15</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>4.17</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.461</v>
+        <v>7.967</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>17.83</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>13.06</v>
+        <v>10.79</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>10.75</v>
+        <v>3.72</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.6</v>
+        <v>1.4</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>4.99</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.528</v>
+        <v>3.489</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13.54</v>
+        <v>114.34</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="n">
-        <v>13</v>
+        <v>-13</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-19.87</v>
+        <v>12.89</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-3.66</v>
+        <v>11.25</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>4.27</v>
+        <v>0.06</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>1.18</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.383</v>
+        <v>0.528</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>110.32</v>
+        <v>13.54</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1144,9 +1142,7 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
         <v>3</v>
@@ -1155,38 +1151,40 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-9.779999999999999</v>
+        <v>-17.87</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.4</v>
+        <v>-3.88</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-0.68</v>
+        <v>2.47</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>2.52</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.376</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>39.07</v>
+        <v>110.32</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1195,31 +1193,31 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-14.58</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-3.85</v>
+        <v>-1.73</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>4.01</v>
+        <v>-0.95</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>0.49</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13">
@@ -1234,7 +1232,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.127</v>
+        <v>3.149</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>21.04</v>
@@ -1249,7 +1247,7 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
@@ -1258,19 +1256,21 @@
         <v>1</v>
       </c>
       <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>3.29</v>
+        <v>4.51</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.45</v>
+        <v>0.79</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.67</v>
+        <v>2.11</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>7.93</v>
+        <v>7.26</v>
       </c>
     </row>
     <row r="14">
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.342</v>
+        <v>0.339</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>108.28</v>
@@ -1318,16 +1318,16 @@
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-9.640000000000001</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-0.45</v>
+        <v>-1.63</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-1.43</v>
+        <v>-0.93</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>4.56</v>
+        <v>2.93</v>
       </c>
     </row>
     <row r="15">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.123</v>
+        <v>1.142</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>41.5</v>
@@ -1357,7 +1357,7 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -1368,19 +1368,21 @@
       <c r="S15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-10.79</v>
+        <v>-8.77</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-11.81</v>
+        <v>-10.56</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>1.8</v>
+        <v>3.25</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>3.13</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="16">
@@ -1395,7 +1397,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.423</v>
+        <v>0.419</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>102.25</v>
@@ -1418,22 +1420,22 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-42.24</v>
+        <v>-42.42</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-17.07</v>
+        <v>-18.02</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1.68</v>
+        <v>-0.84</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-3.38</v>
+        <v>-4.37</v>
       </c>
     </row>
     <row r="17">
@@ -1448,7 +1450,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.172</v>
+        <v>1.204</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>47.73</v>
@@ -1463,7 +1465,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
@@ -1471,20 +1473,24 @@
       <c r="R17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-15.36</v>
+        <v>-12.9</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-4.91</v>
+        <v>-2.64</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>1.22</v>
+        <v>4.62</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-0.73</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="18">
@@ -1499,7 +1505,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.101</v>
+        <v>1.119</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>2.76</v>
@@ -1528,16 +1534,16 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>34.08</v>
+        <v>37.37</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>17.69</v>
+        <v>19.01</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-1.14</v>
+        <v>3.06</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-2.16</v>
+        <v>6.93</v>
       </c>
     </row>
     <row r="19">
@@ -1552,7 +1558,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.829</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>75.37</v>
@@ -1569,32 +1575,28 @@
         <v>-13</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>0.39</v>
+        <v>-0.42</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>2.81</v>
+        <v>4.01</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>-0.83</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-1.2</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="20">
@@ -1609,7 +1611,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.081</v>
+        <v>1.078</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>100.94</v>
@@ -1632,40 +1634,40 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-57.04</v>
+        <v>-55.35</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-19.38</v>
+        <v>-19.75</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-2.01</v>
+        <v>0.08</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-2.69</v>
+        <v>-6.56</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.91</v>
+        <v>2.223</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>49.76</v>
+        <v>40.31</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1677,52 +1679,48 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" s="2" t="inlineStr"/>
-      <c r="U21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-25.03</v>
+        <v>16.87</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-3.41</v>
+        <v>15</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>5</v>
+        <v>1.05</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>5.64</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.235</v>
+        <v>1.05</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>40.31</v>
+        <v>4.63</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1734,7 +1732,7 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
@@ -1746,34 +1744,34 @@
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>14.98</v>
+        <v>45.08</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>16.09</v>
+        <v>21.38</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.95</v>
+        <v>2.53</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>4.38</v>
+        <v>9.630000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.633</v>
+        <v>1.378</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>29.34</v>
+        <v>117.45</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1783,50 +1781,48 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-16.95</v>
+        <v>19.21</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-8.69</v>
+        <v>19.6</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-0.57</v>
+        <v>4.21</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-0.28</v>
+        <v>15.05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.036</v>
+        <v>0.834</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>4.63</v>
+        <v>35.77</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1835,51 +1831,53 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>41.86</v>
+        <v>-22.18</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>20.44</v>
+        <v>-14.76</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-2.75</v>
+        <v>-2</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>7.74</v>
+        <v>-1.49</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.35</v>
+        <v>0.672</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>117.45</v>
+        <v>3.59</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1889,48 +1887,48 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>18.34</v>
+        <v>43.55</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>17.64</v>
+        <v>17.7</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>6.28</v>
+        <v>1.4</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>12.09</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.846</v>
+        <v>2.452</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>35.77</v>
+        <v>35.32</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1939,9 +1937,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
         <v>2</v>
@@ -1949,43 +1945,41 @@
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-20.98</v>
+        <v>-20.6</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-13.24</v>
+        <v>-13.15</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-0.46</v>
+        <v>-3.26</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>2.52</v>
+        <v>-2.14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.668</v>
+        <v>0.973</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>3.59</v>
+        <v>13.22</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1997,48 +1991,48 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>40.61</v>
+        <v>-7.4</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>17.66</v>
+        <v>-4.87</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-2.66</v>
+        <v>2.93</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>9.68</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.483</v>
+        <v>1.777</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>35.32</v>
+        <v>3.16</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2050,46 +2044,48 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S28" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-19.75</v>
+        <v>21.07</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-11.8</v>
+        <v>12.27</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-1.78</v>
+        <v>3.3</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>0.63</v>
+        <v>4.14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.954</v>
+        <v>0.806</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>13.22</v>
+        <v>39.07</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2101,48 +2097,44 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R29" s="2" t="inlineStr"/>
       <c r="S29" s="2" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-9.66</v>
+        <v>-13.1</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-6.44</v>
+        <v>-4.21</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.03</v>
+        <v>1.12</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-0.34</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.756</v>
+        <v>1.894</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3.16</v>
+        <v>49.76</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2154,48 +2146,48 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>18.04</v>
+        <v>-21.95</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>11.46</v>
+        <v>-4.39</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.24</v>
+        <v>2.72</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-1.76</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>3.443</v>
+        <v>1.615</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>10.5</v>
+        <v>29.34</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2207,7 +2199,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2217,16 +2209,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>9.32</v>
+        <v>-16.6</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>3.01</v>
+        <v>-10.03</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-3.78</v>
+        <v>-2.37</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-0.44</v>
+        <v>-2.2</v>
       </c>
     </row>
   </sheetData>
@@ -2257,7 +2249,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-28 | 30 只</t>
+          <t>截至: 2026-08-31 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-01
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.456</v>
+        <v>1.489</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10.5</v>
+        <v>101.66</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,48 +652,46 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R2" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>10.49</v>
+        <v>-9.449999999999999</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.95</v>
+        <v>-2.58</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-1.9</v>
+        <v>-1.56</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-0.08</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.496</v>
+        <v>0.674</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>101.66</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -710,43 +708,45 @@
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-9.01</v>
+        <v>-27.66</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-2.49</v>
+        <v>-10.37</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.24</v>
+        <v>0.74</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-3.13</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.666</v>
+        <v>1.652</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>99.95999999999999</v>
+        <v>101.36</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -756,123 +756,119 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-28.09</v>
+        <v>30.63</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-11.8</v>
+        <v>17.72</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>0.17</v>
+        <v>3.05</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>-2.43</v>
+        <v>10.78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.63</v>
+        <v>0.849</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>101.36</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>29.43</v>
+        <v>-6.7</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>15.88</v>
+        <v>-0.22</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>2.1</v>
+        <v>-3.17</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>8.18</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.848</v>
+        <v>3.055</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>44.27</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
@@ -882,38 +878,42 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-6.08</v>
+        <v>-1.9</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>-0.71</v>
+        <v>1.46</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-1.22</v>
+        <v>1.23</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>1.67</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.041</v>
+        <v>4.684</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>44.27</v>
+        <v>21.63</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -925,12 +925,14 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S7" s="2" t="n">
         <v>1</v>
       </c>
@@ -939,34 +941,34 @@
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-2.55</v>
+        <v>1.14</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.32</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.13</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.685</v>
+        <v>7.881</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>21.63</v>
+        <v>17.83</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -978,125 +980,123 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>0.66</v>
+        <v>11.44</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.05</v>
+        <v>2.84</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.15</v>
+        <v>0.46</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.09</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.967</v>
+        <v>3.482</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>17.83</v>
+        <v>114.34</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>10.79</v>
+        <v>12.87</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>3.72</v>
+        <v>11.33</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>1.4</v>
+        <v>0.87</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>4.46</v>
+        <v>7.94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.489</v>
+        <v>0.378</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>114.34</v>
+        <v>110.32</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L10" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1106,34 +1106,34 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>12.89</v>
+        <v>-8.56</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>11.25</v>
+        <v>-0.83</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.06</v>
+        <v>-2.25</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>5.03</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.528</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13.54</v>
+        <v>39.07</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1145,46 +1145,48 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V11" s="2" t="n">
-        <v>-17.87</v>
+        <v>-11.96</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-3.88</v>
+        <v>-2.4</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>2.47</v>
+        <v>2.62</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.31</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.376</v>
+        <v>3.122</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>110.32</v>
+        <v>21.04</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1193,159 +1195,161 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
       <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-8.539999999999999</v>
+        <v>4.93</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-1.73</v>
+        <v>0.23</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-0.95</v>
+        <v>1.04</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>0.16</v>
+        <v>5.44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.149</v>
+        <v>0.341</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>21.04</v>
+        <v>108.28</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R13" s="2" t="inlineStr"/>
       <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>4.51</v>
+        <v>-8.76</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.79</v>
+        <v>-0.6</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>2.11</v>
+        <v>-2.57</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>7.26</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.339</v>
+        <v>1.141</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>108.28</v>
+        <v>41.5</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-8.710000000000001</v>
+        <v>-7.54</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-1.63</v>
+        <v>-10.31</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-0.93</v>
+        <v>2.83</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.93</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.142</v>
+        <v>0.429</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>41.5</v>
+        <v>102.25</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1355,9 +1359,11 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -1365,42 +1371,44 @@
       <c r="R15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S15" s="2" t="n">
-        <v>1</v>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="T15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-8.77</v>
+        <v>-42.17</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-10.56</v>
+        <v>-15.66</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>3.25</v>
+        <v>1.03</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>2.86</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.419</v>
+        <v>1.197</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>102.25</v>
+        <v>47.73</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1410,50 +1418,50 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-42.42</v>
+        <v>-11.47</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-18.02</v>
+        <v>-2.83</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-0.84</v>
+        <v>3.58</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-4.37</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.204</v>
+        <v>1.091</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>47.73</v>
+        <v>2.76</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1465,50 +1473,46 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-12.9</v>
+        <v>38.62</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-2.64</v>
+        <v>16.16</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>4.62</v>
+        <v>0.14</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>1.54</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.119</v>
+        <v>0.846</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2.76</v>
+        <v>75.37</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1518,9 +1522,11 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -1528,40 +1534,38 @@
       <c r="R18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>37.37</v>
+        <v>-0.39</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>19.01</v>
+        <v>6.5</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>3.06</v>
+        <v>2.09</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>6.93</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.829</v>
+        <v>1.059</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>75.37</v>
+        <v>100.94</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1571,9 +1575,7 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
         <v>2</v>
       </c>
@@ -1581,40 +1583,40 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-0.42</v>
+        <v>-55.29</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>4.01</v>
+        <v>-20.8</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.83</v>
+        <v>-1.36</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-0.48</v>
+        <v>-6.48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.078</v>
+        <v>2.233</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>100.94</v>
+        <v>40.31</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1624,50 +1626,52 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-55.35</v>
+        <v>17.83</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-19.75</v>
+        <v>15.77</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-6.56</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.223</v>
+        <v>1.595</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>40.31</v>
+        <v>29.34</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1679,30 +1683,28 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>16.87</v>
+        <v>-16.6</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>15</v>
+        <v>-10.9</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.05</v>
+        <v>-2.19</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.44</v>
+        <v>-2.67</v>
       </c>
     </row>
     <row r="22">
@@ -1717,7 +1719,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.05</v>
+        <v>1.028</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>4.63</v>
@@ -1741,19 +1743,21 @@
         <v>1</v>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>45.08</v>
+        <v>46.35</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>21.38</v>
+        <v>18.93</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>2.53</v>
+        <v>-0.28</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>9.630000000000001</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="23">
@@ -1768,7 +1772,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.378</v>
+        <v>1.342</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>117.45</v>
@@ -1790,21 +1794,23 @@
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>19.21</v>
+        <v>19.1</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>19.6</v>
+        <v>16.74</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>4.21</v>
+        <v>1.58</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>15.05</v>
+        <v>13.89</v>
       </c>
     </row>
     <row r="24">
@@ -1819,7 +1825,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.834</v>
+        <v>0.826</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>35.77</v>
@@ -1842,24 +1848,22 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="S24" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-22.18</v>
+        <v>-23.97</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-14.76</v>
+        <v>-15.32</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-2</v>
+        <v>-2.35</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-1.49</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="25">
@@ -1874,7 +1878,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.672</v>
+        <v>0.662</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>3.59</v>
@@ -1898,19 +1902,21 @@
         <v>1</v>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>43.55</v>
+        <v>44.84</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>17.7</v>
+        <v>16.05</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.4</v>
+        <v>-0.27</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>8.869999999999999</v>
+        <v>-1.28</v>
       </c>
     </row>
     <row r="26">
@@ -1925,7 +1931,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.452</v>
+        <v>2.416</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>35.32</v>
@@ -1940,7 +1946,7 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
@@ -1952,16 +1958,16 @@
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-20.6</v>
+        <v>-21.59</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-13.15</v>
+        <v>-14.17</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-3.26</v>
+        <v>-2.96</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-2.14</v>
+        <v>-3.17</v>
       </c>
     </row>
     <row r="27">
@@ -1976,7 +1982,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.973</v>
+        <v>0.964</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>13.22</v>
@@ -2002,19 +2008,21 @@
       <c r="S27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-7.4</v>
+        <v>-6.67</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-4.87</v>
+        <v>-5.44</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>2.93</v>
+        <v>0.42</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.61</v>
+        <v>-2.42</v>
       </c>
     </row>
     <row r="28">
@@ -2029,7 +2037,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.777</v>
+        <v>1.74</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3.16</v>
@@ -2049,43 +2057,41 @@
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>21.07</v>
+        <v>22.21</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>12.27</v>
+        <v>10.13</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>3.3</v>
+        <v>0.9</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>4.14</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.806</v>
+        <v>3.412</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>39.07</v>
+        <v>10.5</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2097,7 +2103,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2107,34 +2113,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-13.1</v>
+        <v>10.72</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-4.21</v>
+        <v>1.87</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>1.12</v>
+        <v>-1.98</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-0.88</v>
+        <v>-5.53</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.894</v>
+        <v>0.532</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>49.76</v>
+        <v>13.54</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2146,48 +2152,44 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-21.95</v>
+        <v>-16.49</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-4.39</v>
+        <v>-2.76</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>2.72</v>
+        <v>3.46</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>4.11</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.615</v>
+        <v>1.903</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>29.34</v>
+        <v>49.76</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2199,9 +2201,11 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O31" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
@@ -2209,16 +2213,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-16.6</v>
+        <v>-20.19</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-10.03</v>
+        <v>-3.49</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-2.37</v>
+        <v>3.37</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-2.2</v>
+        <v>6.14</v>
       </c>
     </row>
   </sheetData>
@@ -2249,7 +2253,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-31 | 30 只</t>
+          <t>截至: 2026-09-01 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-02
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.489</v>
+        <v>0.668</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>101.66</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -657,41 +657,43 @@
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>-1</v>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-9.449999999999999</v>
+        <v>-27.27</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-2.58</v>
+        <v>-9.82</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-1.56</v>
+        <v>1.79</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-1.46</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.674</v>
+        <v>1.687</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>99.95999999999999</v>
+        <v>101.36</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -701,166 +703,166 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="Q3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-27.66</v>
+        <v>33.9</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-10.37</v>
+        <v>21.79</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.74</v>
+        <v>13.69</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.45</v>
+        <v>18.69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.652</v>
+        <v>0.843</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>101.36</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>30.63</v>
+        <v>-6.39</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>17.72</v>
+        <v>0.54</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>3.05</v>
+        <v>-1.62</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>10.78</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.849</v>
+        <v>3.025</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>44.27</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-6.7</v>
+        <v>-2.01</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>-0.22</v>
+        <v>1.86</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-3.17</v>
+        <v>1.42</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>0.08</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.055</v>
+        <v>4.62</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44.27</v>
+        <v>21.63</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -877,43 +879,47 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S6" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-1.9</v>
+        <v>0.75</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.46</v>
+        <v>1.33</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>1.23</v>
+        <v>0.2</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.6</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.684</v>
+        <v>7.751</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>21.63</v>
+        <v>17.83</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -923,148 +929,162 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N7" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="2" t="n">
-        <v>1</v>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>1.14</v>
+        <v>11.3</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.32</v>
+        <v>2.52</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.13</v>
+        <v>0.24</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.33</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.881</v>
+        <v>3.428</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>17.83</v>
+        <v>114.34</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R8" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>11.44</v>
+        <v>12.05</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>2.84</v>
+        <v>11.12</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.46</v>
+        <v>0.59</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>2.5</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.482</v>
+        <v>0.521</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>13.54</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="n">
-        <v>-1</v>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>12.87</v>
+        <v>-16.36</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>11.33</v>
+        <v>-3.34</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.87</v>
+        <v>1.03</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>7.94</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="10">
@@ -1079,7 +1099,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.378</v>
+        <v>0.377</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>110.32</v>
@@ -1106,16 +1126,16 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-8.56</v>
+        <v>-8.23</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-0.83</v>
+        <v>0.36</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-2.25</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-0.15</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="11">
@@ -1130,7 +1150,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.805</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>39.07</v>
@@ -1145,12 +1165,16 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr">
@@ -1159,16 +1183,16 @@
         </is>
       </c>
       <c r="V11" s="2" t="n">
-        <v>-11.96</v>
+        <v>-11.97</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-2.4</v>
+        <v>-2.54</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>2.62</v>
+        <v>1.19</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>3.15</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="12">
@@ -1183,7 +1207,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.122</v>
+        <v>3.078</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>21.04</v>
@@ -1198,28 +1222,34 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>4.93</v>
+        <v>4.95</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1.04</v>
+        <v>1.54</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>5.44</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="13">
@@ -1234,7 +1264,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.341</v>
+        <v>0.338</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>108.28</v>
@@ -1267,34 +1297,34 @@
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-8.76</v>
+        <v>-8.609999999999999</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-0.6</v>
+        <v>-0.08</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-2.57</v>
+        <v>-0.71</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>3.34</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.141</v>
+        <v>0.423</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>41.5</v>
+        <v>102.25</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1304,7 +1334,9 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N14" s="2" t="n">
         <v>2</v>
       </c>
@@ -1314,42 +1346,40 @@
       <c r="R14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-7.54</v>
+        <v>-41.73</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-10.31</v>
+        <v>-15.53</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>2.83</v>
+        <v>1.49</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.98</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.429</v>
+        <v>1.177</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>102.25</v>
+        <v>47.73</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1359,56 +1389,50 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-42.17</v>
+        <v>-9.949999999999999</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-15.66</v>
+        <v>-3.08</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>1.03</v>
+        <v>3.93</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>0.3</v>
+        <v>-2.38</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.197</v>
+        <v>1.073</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>47.73</v>
+        <v>2.76</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1420,48 +1444,54 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="n">
-        <v>1</v>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-11.47</v>
+        <v>38.47</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-2.83</v>
+        <v>15.66</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>3.58</v>
+        <v>-0.68</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-5.92</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.091</v>
+        <v>0.844</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2.76</v>
+        <v>75.37</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1471,48 +1501,52 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>38.62</v>
+        <v>-0.62</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>16.16</v>
+        <v>7.77</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>0.14</v>
+        <v>3.17</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>0.13</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.846</v>
+        <v>1.05</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>75.37</v>
+        <v>100.94</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1522,50 +1556,48 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-0.39</v>
+        <v>-55.59</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>6.5</v>
+        <v>-20.25</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>2.09</v>
+        <v>-1.22</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>5.71</v>
+        <v>-5.77</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.059</v>
+        <v>1.852</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>100.94</v>
+        <v>49.76</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1577,28 +1609,34 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-55.29</v>
+        <v>-20.4</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.8</v>
+        <v>-4.62</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-1.36</v>
+        <v>-0.52</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-6.48</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="20">
@@ -1613,7 +1651,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.233</v>
+        <v>2.195</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>40.31</v>
@@ -1633,27 +1671,25 @@
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="T20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>17.83</v>
+        <v>18.47</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>15.77</v>
+        <v>15.3</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.09</v>
+        <v>0.25</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>0.29</v>
+        <v>-2.57</v>
       </c>
     </row>
     <row r="21">
@@ -1668,7 +1704,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.595</v>
+        <v>1.557</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>29.34</v>
@@ -1683,7 +1719,7 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -1695,16 +1731,16 @@
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-16.6</v>
+        <v>-17.89</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-10.9</v>
+        <v>-11.82</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-2.19</v>
+        <v>-3.38</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-2.67</v>
+        <v>-4.38</v>
       </c>
     </row>
     <row r="22">
@@ -1719,7 +1755,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.028</v>
+        <v>1.009</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>4.63</v>
@@ -1734,30 +1770,34 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S22" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>46.35</v>
+        <v>46.32</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>18.93</v>
+        <v>18.13</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.29</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-1</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="23">
@@ -1772,7 +1812,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.342</v>
+        <v>1.303</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>117.45</v>
@@ -1789,7 +1829,7 @@
         <v>-9</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -1797,20 +1837,24 @@
       <c r="R23" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>19.1</v>
+        <v>17.75</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>16.74</v>
+        <v>14.83</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>1.58</v>
+        <v>0.24</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>13.89</v>
+        <v>13.04</v>
       </c>
     </row>
     <row r="24">
@@ -1825,7 +1869,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.826</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>35.77</v>
@@ -1854,16 +1898,16 @@
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-23.97</v>
+        <v>-27.22</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.32</v>
+        <v>-15.68</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-2.35</v>
+        <v>-3.31</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-1.98</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="25">
@@ -1878,7 +1922,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.662</v>
+        <v>0.648</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>3.59</v>
@@ -1899,42 +1943,46 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>44.84</v>
+        <v>44.69</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>16.05</v>
+        <v>14.97</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-0.27</v>
+        <v>-0.13</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-1.28</v>
+        <v>-1.55</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.416</v>
+        <v>0.947</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>35.32</v>
+        <v>13.22</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1951,41 +1999,47 @@
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T26" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-21.59</v>
+        <v>-5.87</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-14.17</v>
+        <v>-5.76</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-2.96</v>
+        <v>1.05</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-3.17</v>
+        <v>-4.16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.964</v>
+        <v>1.708</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>13.22</v>
+        <v>3.16</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1997,50 +2051,54 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S27" s="2" t="n">
-        <v>1</v>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-6.67</v>
+        <v>22.01</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-5.44</v>
+        <v>9.49</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.42</v>
+        <v>-0.48</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-2.42</v>
+        <v>-5.32</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.74</v>
+        <v>3.335</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3.16</v>
+        <v>10.5</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2059,39 +2117,37 @@
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr"/>
-      <c r="T28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>22.21</v>
+        <v>9.85</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>10.13</v>
+        <v>0.89</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>0.9</v>
+        <v>-2.38</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-1.07</v>
+        <v>-6.45</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>3.412</v>
+        <v>1.483</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>10.5</v>
+        <v>101.66</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2103,7 +2159,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2113,34 +2169,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>10.72</v>
+        <v>-10.17</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>1.87</v>
+        <v>-1.61</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-1.98</v>
+        <v>-0.62</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-5.53</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.532</v>
+        <v>1.142</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>13.54</v>
+        <v>41.5</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2152,9 +2208,11 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2162,34 +2220,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-16.49</v>
+        <v>-6.55</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-2.76</v>
+        <v>-8.92</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>3.46</v>
+        <v>4.41</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>2.56</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.903</v>
+        <v>2.364</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>49.76</v>
+        <v>35.32</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2201,11 +2259,9 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
@@ -2213,16 +2269,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-20.19</v>
+        <v>-24.2</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-3.49</v>
+        <v>-14.84</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>3.37</v>
+        <v>-4.13</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>6.14</v>
+        <v>-4.56</v>
       </c>
     </row>
   </sheetData>
@@ -2253,7 +2309,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-01 | 30 只</t>
+          <t>截至: 2026-09-02 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-03
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.668</v>
+        <v>0.665</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>99.95999999999999</v>
@@ -666,16 +666,16 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-27.27</v>
+        <v>-27.83</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-9.82</v>
+        <v>-10.2</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>1.79</v>
+        <v>2.05</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="3">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.687</v>
+        <v>1.664</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>101.36</v>
@@ -703,9 +703,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
         <v>1</v>
       </c>
@@ -714,25 +712,23 @@
       <c r="Q3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>33.9</v>
+        <v>36.43</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>21.79</v>
+        <v>19.92</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>13.69</v>
+        <v>11.9</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>18.69</v>
+        <v>17.27</v>
       </c>
     </row>
     <row r="4">
@@ -747,7 +743,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.843</v>
+        <v>0.851</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>96.56999999999999</v>
@@ -755,20 +751,10 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
@@ -777,21 +763,25 @@
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-6.39</v>
+        <v>-6.49</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.54</v>
+        <v>1.45</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-1.62</v>
+        <v>-0.72</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>0.97</v>
+        <v>3.06</v>
       </c>
     </row>
     <row r="5">
@@ -806,7 +796,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.025</v>
+        <v>3.031</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>44.27</v>
@@ -821,7 +811,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -835,16 +825,16 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-2.01</v>
+        <v>-2.43</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.86</v>
+        <v>1.97</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.42</v>
+        <v>1.48</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>2.7</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="6">
@@ -859,7 +849,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.62</v>
+        <v>4.621</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>21.63</v>
@@ -879,29 +869,25 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R6" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>0.75</v>
+        <v>0.12</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.33</v>
+        <v>1.23</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -916,7 +902,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.751</v>
+        <v>7.781</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>17.83</v>
@@ -933,36 +919,30 @@
         <v>13</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R7" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>11.3</v>
+        <v>10.63</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.52</v>
+        <v>2.77</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.24</v>
+        <v>-1</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.66</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="8">
@@ -977,7 +957,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.428</v>
+        <v>3.436</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>114.34</v>
@@ -1001,7 +981,7 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="n">
-        <v>-13</v>
+        <v>-9</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>
@@ -1012,24 +992,20 @@
       <c r="R8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>12.05</v>
+        <v>11.33</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>11.12</v>
+        <v>11.25</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.59</v>
+        <v>1.23</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>9.25</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="9">
@@ -1044,7 +1020,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.521</v>
+        <v>0.526</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>13.54</v>
@@ -1075,16 +1051,16 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-16.36</v>
+        <v>-16.75</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-3.34</v>
+        <v>-2.41</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>1.03</v>
+        <v>1.59</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>2.54</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="10">
@@ -1099,7 +1075,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.377</v>
+        <v>0.379</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>110.32</v>
@@ -1121,21 +1097,27 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V10" s="2" t="n">
-        <v>-8.23</v>
+        <v>-8.449999999999999</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.36</v>
+        <v>0.87</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.27</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>1.21</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="11">
@@ -1150,7 +1132,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.805</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>39.07</v>
@@ -1165,34 +1147,28 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
       <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="U11" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>-11.97</v>
+        <v>-12.06</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-2.54</v>
+        <v>-0.98</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.19</v>
+        <v>2.91</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>3.75</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="12">
@@ -1207,7 +1183,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.078</v>
+        <v>3.086</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>21.04</v>
@@ -1222,7 +1198,7 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -1232,24 +1208,20 @@
           <t>预-1</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>4.95</v>
+        <v>4.45</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.24</v>
+        <v>0.4</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1.54</v>
+        <v>0.06</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>3.63</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="13">
@@ -1264,7 +1236,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.338</v>
+        <v>0.339</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>108.28</v>
@@ -1273,15 +1245,9 @@
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="n">
         <v>-9</v>
       </c>
@@ -1292,21 +1258,25 @@
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-8.609999999999999</v>
+        <v>-9.01</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-0.08</v>
+        <v>0.18</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.71</v>
+        <v>0.05</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>4.16</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="14">
@@ -1321,7 +1291,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.423</v>
+        <v>0.421</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>102.25</v>
@@ -1343,22 +1313,26 @@
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="n">
-        <v>1</v>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>-41.73</v>
+        <v>-42.65</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-15.53</v>
+        <v>-15.84</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.49</v>
+        <v>2.12</v>
       </c>
       <c r="Y14" s="2" t="n">
         <v>2.09</v>
@@ -1376,7 +1350,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.177</v>
+        <v>1.179</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>47.73</v>
@@ -1391,7 +1365,7 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -1400,21 +1374,19 @@
       <c r="S15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T15" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-9.949999999999999</v>
+        <v>-9.02</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-3.08</v>
+        <v>-2.99</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>3.93</v>
+        <v>1.93</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>-2.38</v>
+        <v>-1.78</v>
       </c>
     </row>
     <row r="16">
@@ -1429,7 +1401,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.073</v>
+        <v>1.066</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>2.76</v>
@@ -1449,31 +1421,23 @@
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>38.47</v>
+        <v>36.83</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>15.66</v>
+        <v>14.62</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-0.68</v>
+        <v>-5.22</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-5.92</v>
+        <v>-8.43</v>
       </c>
     </row>
     <row r="17">
@@ -1488,7 +1452,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.844</v>
+        <v>0.84</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>75.37</v>
@@ -1505,48 +1469,46 @@
         <v>-13</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R17" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-0.62</v>
+        <v>-0.46</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>7.77</v>
+        <v>7.18</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>3.17</v>
+        <v>4.66</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>9.359999999999999</v>
+        <v>8.050000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.05</v>
+        <v>1.871</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>100.94</v>
+        <v>49.76</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1558,9 +1520,11 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O18" s="2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
@@ -1570,34 +1534,34 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-55.59</v>
+        <v>-21.09</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-20.25</v>
+        <v>-3.59</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-1.22</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-5.77</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.852</v>
+        <v>2.196</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>49.76</v>
+        <v>40.31</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1609,52 +1573,46 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-20.4</v>
+        <v>18.36</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-4.62</v>
+        <v>15.14</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.52</v>
+        <v>-0.2</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>5.04</v>
+        <v>-1.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.195</v>
+        <v>1.574</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>40.31</v>
+        <v>29.34</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1666,48 +1624,50 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S20" s="2" t="inlineStr"/>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>18.47</v>
+        <v>-19.1</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>15.3</v>
+        <v>-10.96</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>0.25</v>
+        <v>-1.94</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-2.57</v>
+        <v>-2.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.557</v>
+        <v>1.004</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>29.34</v>
+        <v>4.63</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1719,46 +1679,46 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="n">
+      <c r="R21" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-17.89</v>
+        <v>45.43</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-11.82</v>
+        <v>17.19</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-3.38</v>
+        <v>-4.6</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-4.38</v>
+        <v>-4.22</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.009</v>
+        <v>1.3</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>4.63</v>
+        <v>117.45</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1768,7 +1728,9 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N22" s="2" t="n">
         <v>1</v>
       </c>
@@ -1778,44 +1740,40 @@
       <c r="R22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S22" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>46.32</v>
+        <v>16.07</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>18.13</v>
+        <v>14.38</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.29</v>
+        <v>-2.03</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-1.97</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.303</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>117.45</v>
+        <v>35.77</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1824,55 +1782,51 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L23" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="S23" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
       </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>17.75</v>
+        <v>-29.53</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>14.83</v>
+        <v>-15.86</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>0.24</v>
+        <v>-2.23</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>13.04</v>
+        <v>-1.89</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8110000000000001</v>
+        <v>0.646</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>35.77</v>
+        <v>3.59</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1881,51 +1835,51 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="n">
+      <c r="R24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-27.22</v>
+        <v>43.52</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.68</v>
+        <v>14.28</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-3.31</v>
+        <v>-4.86</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-2.6</v>
+        <v>-3.93</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.648</v>
+        <v>1.703</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>3.59</v>
+        <v>3.16</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1945,44 +1899,38 @@
       <c r="R25" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S25" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T25" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>44.69</v>
+        <v>20.51</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>14.97</v>
+        <v>8.94</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-0.13</v>
+        <v>-4.18</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-1.55</v>
+        <v>-6.38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.947</v>
+        <v>3.33</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>13.22</v>
+        <v>10.5</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1994,52 +1942,44 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-5.87</v>
+        <v>8.76</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-5.76</v>
+        <v>0.57</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1.05</v>
+        <v>-3.57</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-4.16</v>
+        <v>-6.21</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.708</v>
+        <v>1.481</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>3.16</v>
+        <v>101.66</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2051,54 +1991,44 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S27" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>22.01</v>
+        <v>-10.96</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>9.49</v>
+        <v>-1.79</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.48</v>
+        <v>0.48</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-5.32</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>3.335</v>
+        <v>1.14</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>10.5</v>
+        <v>41.5</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2110,9 +2040,11 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
@@ -2120,34 +2052,34 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>9.85</v>
+        <v>-5.79</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>0.89</v>
+        <v>-9.109999999999999</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-2.38</v>
+        <v>3.32</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-6.45</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.483</v>
+        <v>1.035</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>101.66</v>
+        <v>100.94</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2159,7 +2091,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2169,34 +2101,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-10.17</v>
+        <v>-56.64</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-1.61</v>
+        <v>-21.34</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-0.62</v>
+        <v>-1.38</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>0.55</v>
+        <v>-5.09</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.142</v>
+        <v>2.37</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>41.5</v>
+        <v>35.32</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2208,11 +2140,9 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
@@ -2220,34 +2150,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-6.55</v>
+        <v>-26.17</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-8.92</v>
+        <v>-14.71</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>4.41</v>
+        <v>-2.87</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>3.85</v>
+        <v>-3.38</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2.364</v>
+        <v>0.954</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>35.32</v>
+        <v>13.22</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2259,7 +2189,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2269,16 +2199,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-24.2</v>
+        <v>-5.21</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-14.84</v>
+        <v>-5.12</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-4.13</v>
+        <v>0.7</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-4.56</v>
+        <v>-2.88</v>
       </c>
     </row>
   </sheetData>
@@ -2309,7 +2239,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-02 | 30 只</t>
+          <t>截至: 2026-09-03 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-04
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.665</v>
+        <v>1.509</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>99.95999999999999</v>
+        <v>99.02</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,48 +652,46 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-27.83</v>
+        <v>-11.48</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-10.2</v>
+        <v>0.23</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>3.62</v>
+        <v>4.47</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.664</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>101.36</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -705,30 +703,30 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="n">
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>36.43</v>
+        <v>-28.21</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>19.92</v>
+        <v>-7.03</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>11.9</v>
+        <v>3.91</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>17.27</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +741,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.851</v>
+        <v>0.845</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>96.56999999999999</v>
@@ -772,16 +770,16 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-6.49</v>
+        <v>-6.89</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>1.45</v>
+        <v>0.91</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.72</v>
+        <v>-0.28</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>3.06</v>
+        <v>-3.02</v>
       </c>
     </row>
     <row r="5">
@@ -796,7 +794,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.031</v>
+        <v>3.037</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>44.27</v>
@@ -811,7 +809,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -825,16 +823,16 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-2.43</v>
+        <v>-2.63</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.97</v>
+        <v>2.29</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.48</v>
+        <v>1.41</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>2.65</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="6">
@@ -849,10 +847,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.621</v>
+        <v>4.616</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>21.63</v>
+        <v>26.51</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -864,7 +862,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -875,19 +873,21 @@
       <c r="S6" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>0.12</v>
+        <v>-0.41</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.15</v>
+        <v>-0.06</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="7">
@@ -902,10 +902,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.781</v>
+        <v>7.673</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>17.83</v>
+        <v>33.48</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -930,19 +930,21 @@
       <c r="S7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>10.63</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.77</v>
+        <v>1.44</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-1</v>
+        <v>-2.11</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.58</v>
+        <v>-1.74</v>
       </c>
     </row>
     <row r="8">
@@ -957,7 +959,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.436</v>
+        <v>3.438</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>114.34</v>
@@ -989,41 +991,41 @@
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="n">
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>11.33</v>
+        <v>10.87</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>11.25</v>
+        <v>11.4</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>1.23</v>
+        <v>0.65</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>7.3</v>
+        <v>8.550000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.526</v>
+        <v>0.38</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13.54</v>
+        <v>101.49</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1032,53 +1034,55 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V9" s="2" t="n">
-        <v>-16.75</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-2.41</v>
+        <v>1.31</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>1.59</v>
+        <v>0.91</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>4.31</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.379</v>
+        <v>0.823</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>110.32</v>
+        <v>39.07</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1087,55 +1091,49 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="U10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>-8.449999999999999</v>
+        <v>-11.69</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.87</v>
+        <v>-0.2</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.27</v>
+        <v>3.65</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>3.55</v>
+        <v>7.82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8179999999999999</v>
+        <v>3.044</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>39.07</v>
+        <v>45.49</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1147,46 +1145,48 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-12.06</v>
+        <v>3.42</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.9</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>2.91</v>
+        <v>-1.35</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>6.16</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.086</v>
+        <v>0.339</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>21.04</v>
+        <v>106.94</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1195,51 +1195,53 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>4.45</v>
+        <v>-9.43</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.4</v>
+        <v>0.36</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.06</v>
+        <v>0.8</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>3.23</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.339</v>
+        <v>0.434</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>108.28</v>
+        <v>102.25</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1248,53 +1250,53 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-9.01</v>
+        <v>-43.3</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.18</v>
+        <v>-13.06</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.05</v>
+        <v>4.01</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>5.94</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.421</v>
+        <v>1.16</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>102.25</v>
+        <v>47.73</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1304,9 +1306,7 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
         <v>2</v>
       </c>
@@ -1320,40 +1320,36 @@
       </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-42.65</v>
+        <v>-8.460000000000001</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-15.84</v>
+        <v>-4.43</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>2.12</v>
+        <v>0.48</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.09</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.179</v>
+        <v>1.036</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>47.73</v>
+        <v>-0.84</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1365,46 +1361,50 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-9.02</v>
+        <v>35.22</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-2.99</v>
+        <v>11.33</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>1.93</v>
+        <v>-6.36</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>-1.78</v>
+        <v>-14.11</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.066</v>
+        <v>0.848</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>2.76</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1416,46 +1416,46 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>36.83</v>
+        <v>0.46</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>14.62</v>
+        <v>8.35</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-5.22</v>
+        <v>5.54</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-8.43</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.84</v>
+        <v>1.056</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>75.37</v>
+        <v>84.78</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1465,9 +1465,7 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
         <v>2</v>
       </c>
@@ -1475,22 +1473,22 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-0.46</v>
+        <v>-57.55</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>7.18</v>
+        <v>-19.54</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>4.66</v>
+        <v>-0.15</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>8.050000000000001</v>
+        <v>-2.57</v>
       </c>
     </row>
     <row r="18">
@@ -1505,7 +1503,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.871</v>
+        <v>1.907</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>49.76</v>
@@ -1528,22 +1526,22 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-21.09</v>
+        <v>-21.42</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-3.59</v>
+        <v>-1.51</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.9</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>6.98</v>
+        <v>9.609999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1558,10 +1556,10 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.196</v>
+        <v>2.222</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>40.31</v>
+        <v>61.93</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1573,46 +1571,46 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>18.36</v>
+        <v>17.93</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>15.14</v>
+        <v>16.51</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.2</v>
+        <v>0.42</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-1.62</v>
+        <v>-0.21</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.574</v>
+        <v>0.987</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>29.34</v>
+        <v>27.11</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1624,50 +1622,50 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R20" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-19.1</v>
+        <v>44.69</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-10.96</v>
+        <v>15.09</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.94</v>
+        <v>-5.35</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-2.29</v>
+        <v>-8.33</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.004</v>
+        <v>1.298</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4.63</v>
+        <v>117.45</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1677,48 +1675,50 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>45.43</v>
+        <v>14.46</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>17.19</v>
+        <v>14.27</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-4.6</v>
+        <v>-3.38</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>-4.22</v>
+        <v>8.130000000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.3</v>
+        <v>0.639</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>117.45</v>
+        <v>19.95</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1728,11 +1728,9 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
@@ -1740,40 +1738,44 @@
       <c r="R22" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S22" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>16.07</v>
+        <v>42.83</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>14.38</v>
+        <v>12.94</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-2.03</v>
+        <v>-4.72</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>6.47</v>
+        <v>-5.33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>35.77</v>
+        <v>9.44</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1782,51 +1784,51 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S23" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-29.53</v>
+        <v>-5.11</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-15.86</v>
+        <v>-6.58</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-2.23</v>
+        <v>-0.14</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-1.89</v>
+        <v>-4.59</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.646</v>
+        <v>1.668</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>3.59</v>
+        <v>-3.85</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1838,7 +1840,7 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
@@ -1846,40 +1848,42 @@
       <c r="R24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>43.52</v>
+        <v>19.07</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>14.28</v>
+        <v>6.7</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-4.86</v>
+        <v>-4.76</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-3.93</v>
+        <v>-10.31</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.703</v>
+        <v>3.305</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>3.16</v>
+        <v>12.25</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1891,46 +1895,44 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>20.51</v>
+        <v>7.72</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>8.94</v>
+        <v>-0.15</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-4.18</v>
+        <v>-3.16</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-6.38</v>
+        <v>-7.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>3.33</v>
+        <v>1.672</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>10.5</v>
+        <v>101.36</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1952,34 +1954,34 @@
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>8.76</v>
+        <v>38.7</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>0.57</v>
+        <v>20.53</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-3.57</v>
+        <v>9.83</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-6.21</v>
+        <v>17.74</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.481</v>
+        <v>0.528</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>101.66</v>
+        <v>13.54</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1991,9 +1993,11 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O27" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
@@ -2001,16 +2005,16 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-10.96</v>
+        <v>-16.86</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-1.79</v>
+        <v>-1.85</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.48</v>
+        <v>1.81</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>2.11</v>
+        <v>5.64</v>
       </c>
     </row>
     <row r="28">
@@ -2025,10 +2029,10 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.14</v>
+        <v>1.148</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>41.5</v>
+        <v>33.19</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2042,9 +2046,7 @@
       <c r="N28" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
@@ -2052,34 +2054,34 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-5.79</v>
+        <v>-5.02</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-9.109999999999999</v>
+        <v>-8.33</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>3.32</v>
+        <v>3.48</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>3.56</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.035</v>
+        <v>1.554</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>100.94</v>
+        <v>39.7</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2091,7 +2093,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2101,34 +2103,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-56.64</v>
+        <v>-21.1</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-21.34</v>
+        <v>-12.02</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-1.38</v>
+        <v>-3.33</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-5.09</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2.37</v>
+        <v>0.805</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>35.32</v>
+        <v>35.77</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2140,7 +2142,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2150,34 +2152,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-26.17</v>
+        <v>-32.54</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-14.71</v>
+        <v>-16.29</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-2.87</v>
+        <v>-3.05</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-3.38</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.954</v>
+        <v>2.349</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>13.22</v>
+        <v>35.32</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2189,7 +2191,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2199,16 +2201,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
+        <v>-28.81</v>
+      </c>
+      <c r="W31" s="2" t="n">
+        <v>-15.45</v>
+      </c>
+      <c r="X31" s="2" t="n">
+        <v>-3.64</v>
+      </c>
+      <c r="Y31" s="2" t="n">
         <v>-5.21</v>
-      </c>
-      <c r="W31" s="2" t="n">
-        <v>-5.12</v>
-      </c>
-      <c r="X31" s="2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="Y31" s="2" t="n">
-        <v>-2.88</v>
       </c>
     </row>
   </sheetData>
@@ -2239,7 +2241,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-03 | 30 只</t>
+          <t>截至: 2026-09-04 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-06
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -706,9 +706,7 @@
         <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="n">
@@ -2365,14 +2363,14 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5%。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=1.8x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-07
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.509</v>
+        <v>3.414</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>99.02</v>
+        <v>12.25</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,7 +652,7 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
@@ -664,34 +664,34 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-11.48</v>
+        <v>7.66</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.23</v>
+        <v>2.45</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>2</v>
+        <v>-0.5</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>4.47</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.6870000000000001</v>
+        <v>1.495</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>95.98999999999999</v>
+        <v>99.02</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -703,46 +703,46 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-28.21</v>
+        <v>-12.55</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-7.03</v>
+        <v>-1.26</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>3.91</v>
+        <v>1.22</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>7.08</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.845</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -754,30 +754,28 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-6.89</v>
+        <v>-28.67</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.91</v>
+        <v>-8.02</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.28</v>
+        <v>3.78</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>-3.02</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="5">
@@ -792,7 +790,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.037</v>
+        <v>3.018</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>44.27</v>
@@ -812,25 +810,23 @@
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R5" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-2.63</v>
+        <v>-3.21</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>2.29</v>
+        <v>1.05</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.41</v>
+        <v>0.36</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>2.64</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="6">
@@ -845,7 +841,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.616</v>
+        <v>4.634</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>26.51</v>
@@ -860,7 +856,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -868,24 +864,22 @@
       <c r="R6" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S6" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-0.41</v>
+        <v>-0.85</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.01</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.03</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.13</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -900,7 +894,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.673</v>
+        <v>7.771</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>33.48</v>
@@ -933,16 +927,16 @@
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>9.539999999999999</v>
+        <v>8.82</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.44</v>
+        <v>2.08</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-2.11</v>
+        <v>-1.64</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-1.74</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="8">
@@ -957,7 +951,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.438</v>
+        <v>3.39</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>114.34</v>
@@ -993,37 +987,39 @@
       <c r="S8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>10.87</v>
+        <v>9.76</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>11.4</v>
+        <v>9.18</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.65</v>
+        <v>-2.07</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>8.550000000000001</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.38</v>
+        <v>0.523</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>101.49</v>
+        <v>13.54</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1032,9 +1028,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
         <v>3</v>
@@ -1043,44 +1037,40 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-8.800000000000001</v>
+        <v>-17.01</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>1.31</v>
+        <v>-3.25</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.91</v>
+        <v>0.63</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>0.53</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.823</v>
+        <v>0.378</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>39.07</v>
+        <v>101.49</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1089,49 +1079,51 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-11.69</v>
+        <v>-8.880000000000001</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-0.2</v>
+        <v>0.24</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>3.65</v>
+        <v>1.97</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>7.82</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3.044</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45.49</v>
+        <v>39.07</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1151,40 +1143,40 @@
       <c r="R11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S11" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V11" s="2" t="n">
-        <v>3.42</v>
+        <v>-12.03</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-0.9</v>
+        <v>-2.65</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-1.35</v>
+        <v>1.56</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.89</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.339</v>
+        <v>3.097</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>106.94</v>
+        <v>45.49</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1193,12 +1185,10 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -1208,38 +1198,42 @@
           <t>预1</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-9.43</v>
+        <v>2.92</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.36</v>
+        <v>0.26</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.8</v>
+        <v>-0.54</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>2.66</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.434</v>
+        <v>0.337</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>102.25</v>
+        <v>106.94</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1248,53 +1242,49 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="L13" s="2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-43.3</v>
+        <v>-9.83</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-13.06</v>
+        <v>-0.72</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>4.01</v>
+        <v>0.91</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>5.27</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.16</v>
+        <v>1.151</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>47.73</v>
+        <v>33.19</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1304,50 +1294,50 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-8.460000000000001</v>
+        <v>-4.38</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-4.43</v>
+        <v>-8.58</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>0.48</v>
+        <v>1.98</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>-2.6</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.036</v>
+        <v>0.433</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>-0.84</v>
+        <v>102.25</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1357,52 +1347,52 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R15" s="2" t="inlineStr"/>
       <c r="S15" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>35.22</v>
+        <v>-43.88</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>11.33</v>
+        <v>-13.58</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-6.36</v>
+        <v>4.44</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>-14.11</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.848</v>
+        <v>1.164</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>97.68000000000001</v>
+        <v>47.73</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1414,46 +1404,46 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>0.46</v>
+        <v>-8.460000000000001</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>8.35</v>
+        <v>-4.64</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>5.54</v>
+        <v>-2.01</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>10.9</v>
+        <v>-2.24</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.056</v>
+        <v>1.062</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>84.78</v>
+        <v>-0.84</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1465,46 +1455,52 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-57.55</v>
+        <v>33.76</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-19.54</v>
+        <v>13.31</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-0.15</v>
+        <v>-5.7</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-2.57</v>
+        <v>-11.01</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.907</v>
+        <v>0.835</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>49.76</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1516,48 +1512,46 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-21.42</v>
+        <v>0.39</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-1.51</v>
+        <v>6.08</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>1.9</v>
+        <v>2.07</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>9.609999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.222</v>
+        <v>1.049</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>61.93</v>
+        <v>84.78</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1569,7 +1563,7 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -1581,34 +1575,34 @@
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>17.93</v>
+        <v>-58.84</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>16.51</v>
+        <v>-20.42</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.42</v>
+        <v>-0.67</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-0.21</v>
+        <v>-4.51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.987</v>
+        <v>1.879</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>27.11</v>
+        <v>49.76</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1620,50 +1614,50 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S20" s="2" t="n">
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
         <v>-1</v>
-      </c>
-      <c r="T20" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>44.69</v>
+        <v>-22.18</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>15.09</v>
+        <v>-3.39</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-5.35</v>
+        <v>1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-8.33</v>
+        <v>6.57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.298</v>
+        <v>2.236</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>117.45</v>
+        <v>61.93</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1674,49 +1668,55 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="n">
+      <c r="R21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>14.46</v>
+        <v>17.27</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>14.27</v>
+        <v>16.44</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-3.38</v>
+        <v>1.44</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>8.130000000000001</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.639</v>
+        <v>1.049</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>19.95</v>
+        <v>27.11</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1728,52 +1728,50 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S22" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="T22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>42.83</v>
+        <v>45.08</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>12.94</v>
+        <v>21.34</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-4.72</v>
+        <v>-0.03</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-5.33</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9379999999999999</v>
+        <v>1.27</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>9.44</v>
+        <v>117.45</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1783,50 +1781,52 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N23" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>-5.11</v>
+        <v>12.38</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>-6.58</v>
+        <v>11.06</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-0.14</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-4.59</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.668</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>-3.85</v>
+        <v>35.77</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1838,50 +1838,48 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S24" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T24" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>19.07</v>
+        <v>-32.65</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>6.7</v>
+        <v>-15.43</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-4.76</v>
+        <v>-0.67</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-10.31</v>
+        <v>-2.23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>3.305</v>
+        <v>0.677</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>12.25</v>
+        <v>19.95</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1893,44 +1891,46 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>7.72</v>
+        <v>43.29</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-0.15</v>
+        <v>18.71</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-3.16</v>
+        <v>1.01</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-7.2</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.672</v>
+        <v>2.373</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>101.36</v>
+        <v>35.32</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1942,44 +1942,48 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>38.7</v>
+        <v>-29.38</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>20.53</v>
+        <v>-15.14</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>9.83</v>
+        <v>-1.99</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>17.74</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.528</v>
+        <v>0.956</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>13.54</v>
+        <v>9.44</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1991,46 +1995,50 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr"/>
-      <c r="T27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-16.86</v>
+        <v>-4.89</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-1.85</v>
+        <v>-5.31</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>1.81</v>
+        <v>-0.44</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>5.64</v>
+        <v>-2.21</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.148</v>
+        <v>1.705</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>33.19</v>
+        <v>-3.85</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2042,44 +2050,52 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
-      <c r="T28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-5.02</v>
+        <v>18.09</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-8.33</v>
+        <v>8.34</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>3.48</v>
+        <v>-3.93</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>3.65</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.554</v>
+        <v>1.679</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>39.7</v>
+        <v>101.36</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2091,7 +2107,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2101,34 +2117,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-21.1</v>
+        <v>39.56</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-12.02</v>
+        <v>20.22</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-3.33</v>
+        <v>4.34</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-3.7</v>
+        <v>17.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.805</v>
+        <v>0.841</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>35.77</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2150,34 +2166,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-32.54</v>
+        <v>-7.36</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-16.29</v>
+        <v>-0.09</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-3.05</v>
+        <v>0.62</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-3.64</v>
+        <v>-4.93</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2.349</v>
+        <v>1.558</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>35.32</v>
+        <v>39.7</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2199,16 +2215,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-28.81</v>
+        <v>-21.98</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-15.45</v>
+        <v>-12.33</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-3.64</v>
+        <v>-2.3</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-5.21</v>
+        <v>-4.88</v>
       </c>
     </row>
   </sheetData>
@@ -2239,7 +2255,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-04 | 30 只</t>
+          <t>截至: 2026-09-07 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-08
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.414</v>
+        <v>3.376</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -664,16 +664,16 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>7.66</v>
+        <v>7.53</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.45</v>
+        <v>1.6</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-0.5</v>
+        <v>-0.27</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-3.5</v>
+        <v>-5.28</v>
       </c>
     </row>
     <row r="3">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.495</v>
+        <v>1.486</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>99.02</v>
@@ -703,28 +703,30 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="n">
-        <v>1</v>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-12.55</v>
+        <v>-13.32</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-1.26</v>
+        <v>-1.44</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.22</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="4">
@@ -766,34 +768,34 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-28.67</v>
+        <v>-29.51</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-8.02</v>
+        <v>-7.58</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>3.78</v>
+        <v>2.79</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>3.82</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.018</v>
+        <v>0.849</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>44.27</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
@@ -811,40 +813,40 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-3.21</v>
+        <v>-7.98</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.05</v>
+        <v>1.28</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>0.36</v>
+        <v>1.5</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>1.26</v>
+        <v>-4.81</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.634</v>
+        <v>3.017</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>26.51</v>
+        <v>44.27</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -856,7 +858,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -870,16 +872,16 @@
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-0.85</v>
+        <v>-3.8</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.01</v>
+        <v>1.4</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.06</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="7">
@@ -894,7 +896,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.771</v>
+        <v>7.788</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>33.48</v>
@@ -916,27 +918,29 @@
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S7" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>8.82</v>
+        <v>8.48</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.08</v>
+        <v>2.63</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-1.64</v>
+        <v>-0.21</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-1.53</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="8">
@@ -951,7 +955,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.39</v>
+        <v>3.446</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>114.34</v>
@@ -983,7 +987,11 @@
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="n">
         <v>-1</v>
       </c>
@@ -992,16 +1000,16 @@
       </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>9.76</v>
+        <v>9.19</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>9.18</v>
+        <v>11.35</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-2.07</v>
+        <v>0.01</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>5.31</v>
+        <v>6.91</v>
       </c>
     </row>
     <row r="9">
@@ -1016,7 +1024,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.523</v>
+        <v>0.52</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>13.54</v>
@@ -1039,20 +1047,26 @@
       <c r="R9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-17.01</v>
+        <v>-17.41</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-3.25</v>
+        <v>-3.37</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.63</v>
+        <v>-0.6</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>4.12</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="10">
@@ -1067,7 +1081,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.378</v>
+        <v>0.379</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>101.49</v>
@@ -1089,23 +1103,25 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="V10" s="2" t="n">
-        <v>-8.880000000000001</v>
+        <v>-9.289999999999999</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.24</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>1.97</v>
+        <v>1.76</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-2.78</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="11">
@@ -1120,7 +1136,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.801</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>39.07</v>
@@ -1135,7 +1151,7 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
@@ -1143,22 +1159,24 @@
       <c r="R11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-12.03</v>
+        <v>-12.85</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-2.65</v>
+        <v>-2.96</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>1.56</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>5.32</v>
+        <v>5.07</v>
       </c>
     </row>
     <row r="12">
@@ -1173,7 +1191,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.097</v>
+        <v>3.106</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>45.49</v>
@@ -1199,23 +1217,25 @@
         </is>
       </c>
       <c r="S12" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V12" s="2" t="n">
-        <v>2.92</v>
+        <v>2.64</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.26</v>
+        <v>0.87</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-0.54</v>
+        <v>0.64</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>1.62</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="13">
@@ -1230,7 +1250,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.337</v>
+        <v>0.341</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>106.94</v>
@@ -1252,21 +1272,23 @@
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-9.83</v>
+        <v>-10.3</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-0.72</v>
+        <v>0.93</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.91</v>
+        <v>1.54</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-0.33</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="14">
@@ -1281,7 +1303,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.151</v>
+        <v>1.162</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>33.19</v>
@@ -1298,7 +1320,7 @@
         <v>-9</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>1</v>
@@ -1308,18 +1330,22 @@
       <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>-4.38</v>
+        <v>-3.49</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-8.58</v>
+        <v>-7.33</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.98</v>
+        <v>2.98</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.12</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="15">
@@ -1334,7 +1360,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.433</v>
+        <v>0.432</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>102.25</v>
@@ -1347,9 +1373,7 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
@@ -1365,16 +1389,16 @@
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-43.88</v>
+        <v>-45.22</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-13.58</v>
+        <v>-13.35</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>4.44</v>
+        <v>2.3</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>2.85</v>
+        <v>3.04</v>
       </c>
     </row>
     <row r="16">
@@ -1389,7 +1413,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.164</v>
+        <v>1.145</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>47.73</v>
@@ -1404,7 +1428,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1412,20 +1436,24 @@
       <c r="R16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-8.460000000000001</v>
+        <v>-8.67</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-4.64</v>
+        <v>-5.74</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-2.01</v>
+        <v>-2.91</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-2.24</v>
+        <v>-3.43</v>
       </c>
     </row>
     <row r="17">
@@ -1440,7 +1468,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.062</v>
+        <v>1.048</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>-0.84</v>
@@ -1460,29 +1488,23 @@
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R17" s="2" t="inlineStr"/>
       <c r="S17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T17" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>33.76</v>
+        <v>33.07</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>13.31</v>
+        <v>12.07</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-5.7</v>
+        <v>-4.1</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-11.01</v>
+        <v>-11.42</v>
       </c>
     </row>
     <row r="18">
@@ -1497,7 +1519,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.835</v>
+        <v>0.839</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>97.68000000000001</v>
@@ -1524,16 +1546,16 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>0.39</v>
+        <v>-0.16</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>6.08</v>
+        <v>6.99</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>2.07</v>
+        <v>0.49</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>8.1</v>
+        <v>8.49</v>
       </c>
     </row>
     <row r="19">
@@ -1548,7 +1570,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.049</v>
+        <v>1.042</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>84.78</v>
@@ -1563,28 +1585,30 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="n">
-        <v>1</v>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-58.84</v>
+        <v>-59.59</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.42</v>
+        <v>-20.54</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-0.67</v>
+        <v>0.26</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-4.51</v>
+        <v>-4.35</v>
       </c>
     </row>
     <row r="20">
@@ -1599,7 +1623,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.879</v>
+        <v>1.846</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>49.76</v>
@@ -1624,22 +1648,24 @@
       <c r="R20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T20" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-22.18</v>
+        <v>-23.18</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-3.39</v>
+        <v>-4.62</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>1</v>
+        <v>-1.13</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>6.57</v>
+        <v>5.44</v>
       </c>
     </row>
     <row r="21">
@@ -1654,7 +1680,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.236</v>
+        <v>2.233</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>61.93</v>
@@ -1679,26 +1705,22 @@
       <c r="R21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>17.27</v>
+        <v>16.92</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>16.44</v>
+        <v>16.58</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.44</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>0.25</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="22">
@@ -1713,7 +1735,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.049</v>
+        <v>1.042</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>27.11</v>
@@ -1728,7 +1750,7 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
@@ -1739,21 +1761,19 @@
       <c r="S22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T22" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>45.08</v>
+        <v>46.47</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>21.34</v>
+        <v>20.72</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.03</v>
+        <v>1.78</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>1.25</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="23">
@@ -1768,7 +1788,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.27</v>
+        <v>1.302</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>117.45</v>
@@ -1785,30 +1805,32 @@
         <v>-9</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>12.38</v>
+        <v>11.72</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>11.06</v>
+        <v>14.19</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-8.539999999999999</v>
+        <v>-2.56</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>2.68</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="24">
@@ -1823,7 +1845,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.819</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>35.77</v>
@@ -1843,25 +1865,27 @@
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
+      <c r="R24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
-      <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-32.65</v>
+        <v>-32.64</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.43</v>
+        <v>-15.01</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.67</v>
+        <v>0.3</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-2.23</v>
+        <v>-3.12</v>
       </c>
     </row>
     <row r="25">
@@ -1876,7 +1900,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.677</v>
+        <v>0.671</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>19.95</v>
@@ -1903,16 +1927,16 @@
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>43.29</v>
+        <v>44.55</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>18.71</v>
+        <v>17.85</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.01</v>
+        <v>1.79</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>3.77</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="26">
@@ -1927,7 +1951,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.373</v>
+        <v>2.362</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>35.32</v>
@@ -1940,7 +1964,9 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N26" s="2" t="n">
         <v>1</v>
       </c>
@@ -1956,16 +1982,16 @@
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-29.38</v>
+        <v>-30.54</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-15.14</v>
+        <v>-15.2</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-1.99</v>
+        <v>-1.03</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-5.3</v>
+        <v>-6.07</v>
       </c>
     </row>
     <row r="27">
@@ -1980,7 +2006,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.956</v>
+        <v>0.951</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>9.44</v>
@@ -2001,7 +2027,7 @@
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S27" s="2" t="n">
         <v>1</v>
@@ -2011,16 +2037,16 @@
       </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-4.89</v>
+        <v>-4.26</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-5.31</v>
+        <v>-5.44</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.44</v>
+        <v>-0</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-2.21</v>
+        <v>-4.09</v>
       </c>
     </row>
     <row r="28">
@@ -2035,7 +2061,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.705</v>
+        <v>1.681</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>-3.85</v>
@@ -2055,29 +2081,23 @@
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T28" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>18.09</v>
+        <v>17.77</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>8.34</v>
+        <v>7.12</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-3.93</v>
+        <v>-3.01</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-8</v>
+        <v>-8.16</v>
       </c>
     </row>
     <row r="29">
@@ -2092,7 +2112,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.679</v>
+        <v>1.748</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>101.36</v>
@@ -2117,34 +2137,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>39.56</v>
+        <v>41.39</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>20.22</v>
+        <v>25.47</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>4.34</v>
+        <v>7.75</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>17.55</v>
+        <v>18.83</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.841</v>
+        <v>4.624</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>26.51</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2156,7 +2176,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2166,16 +2186,16 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-7.36</v>
+        <v>-1.22</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-0.09</v>
+        <v>1.14</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>0.62</v>
+        <v>-0.18</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-4.93</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="31">
@@ -2190,7 +2210,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.558</v>
+        <v>1.542</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>39.7</v>
@@ -2215,16 +2235,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-21.98</v>
+        <v>-23.91</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-12.33</v>
+        <v>-12.94</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-2.3</v>
+        <v>-2.04</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-4.88</v>
+        <v>-5.49</v>
       </c>
     </row>
   </sheetData>
@@ -2255,7 +2275,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-07 | 30 只</t>
+          <t>截至: 2026-09-08 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-09
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.376</v>
+        <v>3.373</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>12.25</v>
@@ -664,16 +664,16 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>7.53</v>
+        <v>8.5</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.6</v>
+        <v>1.14</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-0.27</v>
+        <v>0.24</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-5.28</v>
+        <v>-6.69</v>
       </c>
     </row>
     <row r="3">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.486</v>
+        <v>1.481</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>99.02</v>
@@ -708,25 +708,23 @@
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R3" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-13.32</v>
+        <v>-13.73</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-1.44</v>
+        <v>-2.08</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>1.14</v>
+        <v>-0.47</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.79</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="4">
@@ -741,7 +739,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.679</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>95.98999999999999</v>
@@ -756,28 +754,30 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-29.51</v>
+        <v>-29.86</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-7.58</v>
+        <v>-8.289999999999999</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>2.79</v>
+        <v>1.52</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>4.58</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="5">
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.849</v>
+        <v>0.837</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>96.56999999999999</v>
@@ -813,22 +813,22 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-7.98</v>
+        <v>-8.92</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>1.28</v>
+        <v>-0.38</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.5</v>
+        <v>-0.92</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-4.81</v>
+        <v>-5.59</v>
       </c>
     </row>
     <row r="6">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.017</v>
+        <v>3.021</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>44.27</v>
@@ -875,31 +875,31 @@
         <v>-3.8</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.4</v>
+        <v>1.24</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.61</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>1.94</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.788</v>
+        <v>4.637</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>33.48</v>
+        <v>26.51</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -909,11 +909,9 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -931,55 +929,45 @@
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>8.48</v>
+        <v>-0.83</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.63</v>
+        <v>1.12</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.21</v>
+        <v>-0.2</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-1.16</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.446</v>
+        <v>7.785</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>114.34</v>
+        <v>33.48</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>
@@ -992,99 +980,105 @@
           <t>预1</t>
         </is>
       </c>
-      <c r="S8" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>9.19</v>
+        <v>8.92</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>11.35</v>
+        <v>2.24</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.28</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>6.91</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.52</v>
+        <v>3.498</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13.54</v>
+        <v>114.34</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N9" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>-1</v>
-      </c>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-17.41</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-3.37</v>
+        <v>12.64</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-0.6</v>
+        <v>1.52</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>3.68</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.379</v>
+        <v>0.518</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>101.49</v>
+        <v>13.54</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1093,9 +1087,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
         <v>3</v>
@@ -1103,43 +1095,43 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="T10" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-9.289999999999999</v>
+        <v>-17.28</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>-3.93</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>1.76</v>
+        <v>-0.59</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-2.46</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.801</v>
+        <v>0.374</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>39.07</v>
+        <v>101.49</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1148,10 +1140,12 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
@@ -1159,42 +1153,38 @@
       <c r="R11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-12.85</v>
+        <v>-9.99</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-2.96</v>
+        <v>-0.66</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-1.02</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>5.07</v>
+        <v>-3.02</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.106</v>
+        <v>0.802</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>45.49</v>
+        <v>39.07</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1206,54 +1196,46 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>2.64</v>
+        <v>-13.01</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.87</v>
+        <v>-3.06</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.64</v>
+        <v>-0.51</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>1.77</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.341</v>
+        <v>3.101</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>106.94</v>
+        <v>45.49</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1262,51 +1244,51 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V13" s="2" t="n">
-        <v>-10.3</v>
+        <v>2.96</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.93</v>
+        <v>0.38</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.54</v>
+        <v>0.15</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>0.99</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.162</v>
+        <v>0.337</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>33.19</v>
+        <v>106.94</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1315,55 +1297,53 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
+      <c r="L14" s="2" t="n">
         <v>-9</v>
       </c>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-3.49</v>
+        <v>-10.7</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-7.33</v>
+        <v>-0.53</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>2.98</v>
+        <v>-0.45</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>4.44</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.432</v>
+        <v>1.18</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>102.25</v>
+        <v>33.19</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1373,9 +1353,11 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>1</v>
@@ -1383,40 +1365,40 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="n">
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-45.22</v>
+        <v>-2.31</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-13.35</v>
+        <v>-6.14</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.3</v>
+        <v>2.78</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>3.04</v>
+        <v>5.47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.145</v>
+        <v>0.426</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>47.73</v>
+        <v>102.25</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1428,50 +1410,52 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>-1</v>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S16" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T16" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-8.67</v>
+        <v>-46.19</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-5.74</v>
+        <v>-14.67</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-2.91</v>
+        <v>0.86</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-3.43</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.048</v>
+        <v>1.135</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-0.84</v>
+        <v>47.73</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1483,28 +1467,32 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>33.07</v>
+        <v>-8.5</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>12.07</v>
+        <v>-6.79</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-4.1</v>
+        <v>-3.71</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-11.42</v>
+        <v>-3.93</v>
       </c>
     </row>
     <row r="18">
@@ -1519,7 +1507,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.839</v>
+        <v>0.842</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>97.68000000000001</v>
@@ -1539,23 +1527,25 @@
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="n">
-        <v>-1</v>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.68</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>6.99</v>
+        <v>7.07</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>0.49</v>
+        <v>-0.7</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>8.49</v>
+        <v>9.06</v>
       </c>
     </row>
     <row r="19">
@@ -1570,7 +1560,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.042</v>
+        <v>1.029</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>84.78</v>
@@ -1585,30 +1575,28 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R19" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-59.59</v>
+        <v>-60.02</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.54</v>
+        <v>-21.64</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.26</v>
+        <v>-1.39</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-4.35</v>
+        <v>-3.29</v>
       </c>
     </row>
     <row r="20">
@@ -1638,7 +1626,7 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>1</v>
@@ -1651,21 +1639,19 @@
       <c r="S20" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T20" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-23.18</v>
+        <v>-23.05</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-4.62</v>
+        <v>-4.79</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.13</v>
+        <v>-0.17</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>5.44</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="21">
@@ -1680,7 +1666,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.233</v>
+        <v>2.234</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>61.93</v>
@@ -1702,43 +1688,41 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>16.92</v>
+        <v>17.43</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>16.58</v>
+        <v>16.16</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.89</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.042</v>
+        <v>1.542</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>27.11</v>
+        <v>39.7</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1750,48 +1734,48 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>46.47</v>
+        <v>-24.31</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>20.72</v>
+        <v>-13.21</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.78</v>
+        <v>-1.4</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>0.17</v>
+        <v>-5.86</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.302</v>
+        <v>1.052</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>117.45</v>
+        <v>27.11</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1801,54 +1785,50 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>11.72</v>
+        <v>48.96</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>14.19</v>
+        <v>21.26</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>-2.56</v>
+        <v>3.13</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>5.06</v>
+        <v>-1.95</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.819</v>
+        <v>1.341</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>35.77</v>
+        <v>117.45</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1858,52 +1838,52 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S24" s="2" t="inlineStr">
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>预1</t>
         </is>
       </c>
+      <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-32.64</v>
+        <v>13.08</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.01</v>
+        <v>17.14</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>0.3</v>
+        <v>2.31</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-3.12</v>
+        <v>9.77</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.671</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>19.95</v>
+        <v>35.77</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1915,7 +1895,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -1927,34 +1907,34 @@
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>44.55</v>
+        <v>-31.62</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>17.85</v>
+        <v>-15.47</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.79</v>
+        <v>0.21</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>1.88</v>
+        <v>-4.47</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.362</v>
+        <v>0.677</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>35.32</v>
+        <v>19.95</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1964,52 +1944,48 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R26" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-30.54</v>
+        <v>47.02</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-15.2</v>
+        <v>18.31</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-1.03</v>
+        <v>3.34</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-6.07</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.951</v>
+        <v>2.362</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>9.44</v>
+        <v>35.32</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -2019,52 +1995,50 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T27" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-4.26</v>
+        <v>-30.32</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-5.44</v>
+        <v>-15.46</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0</v>
+        <v>-0.62</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-4.09</v>
+        <v>-6.57</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.681</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>-3.85</v>
+        <v>9.44</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2076,28 +2050,30 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S28" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>17.77</v>
+        <v>-3.55</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>7.12</v>
+        <v>-6.58</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-3.01</v>
+        <v>-0.82</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-8.16</v>
+        <v>-4.19</v>
       </c>
     </row>
     <row r="29">
@@ -2112,7 +2088,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.748</v>
+        <v>1.756</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>101.36</v>
@@ -2127,7 +2103,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2137,34 +2113,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>41.39</v>
+        <v>42.77</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>25.47</v>
+        <v>25.52</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>7.75</v>
+        <v>3.73</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>18.83</v>
+        <v>20.54</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>4.624</v>
+        <v>1.043</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>26.51</v>
+        <v>-0.84</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2186,34 +2162,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-1.22</v>
+        <v>33.12</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>1.14</v>
+        <v>11.05</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-0.18</v>
+        <v>-4.6</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-0.1</v>
+        <v>-13.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.542</v>
+        <v>1.671</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>39.7</v>
+        <v>-3.85</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2225,7 +2201,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2235,16 +2211,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>-23.91</v>
+        <v>18.06</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>-12.94</v>
+        <v>6.08</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-2.04</v>
+        <v>-3.41</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-5.49</v>
+        <v>-10.08</v>
       </c>
     </row>
   </sheetData>
@@ -2275,7 +2251,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-08 | 30 只</t>
+          <t>截至: 2026-09-09 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-10
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.373</v>
+        <v>1.466</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>12.25</v>
+        <v>99.02</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,46 +652,46 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>8.5</v>
+        <v>-13.69</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.14</v>
+        <v>-2.47</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.24</v>
+        <v>-0.68</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-6.69</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.481</v>
+        <v>0.667</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>99.02</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -711,38 +711,42 @@
       <c r="R3" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-13.73</v>
+        <v>-29.43</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-2.08</v>
+        <v>-9.32</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-0.47</v>
+        <v>0.88</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.62</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.679</v>
+        <v>1.769</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>95.98999999999999</v>
+        <v>101.36</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -752,9 +756,11 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -768,16 +774,16 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-29.86</v>
+        <v>44.95</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-8.289999999999999</v>
+        <v>26.98</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>1.52</v>
+        <v>7.05</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>4.02</v>
+        <v>20.88</v>
       </c>
     </row>
     <row r="5">
@@ -792,7 +798,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.837</v>
+        <v>0.821</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>96.56999999999999</v>
@@ -807,7 +813,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -819,16 +825,16 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-8.92</v>
+        <v>-9.82</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>-0.38</v>
+        <v>-1.7</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-0.92</v>
+        <v>-3.16</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-5.59</v>
+        <v>-8.720000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -843,7 +849,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.021</v>
+        <v>3.016</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>44.27</v>
@@ -858,48 +864,46 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.8</v>
+        <v>-3.58</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.24</v>
+        <v>1.61</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.61</v>
+        <v>-0.36</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.2</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.637</v>
+        <v>7.742</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26.51</v>
+        <v>33.48</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -909,176 +913,162 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N7" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-0.83</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>1.12</v>
+        <v>2.17</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.6</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.05</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.785</v>
+        <v>3.473</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>33.48</v>
+        <v>114.34</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>8.92</v>
+        <v>10.13</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>2.24</v>
+        <v>12.39</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-0.28</v>
+        <v>1.14</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-1.73</v>
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.498</v>
+        <v>0.369</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>114.34</v>
+        <v>101.49</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>-9</v>
       </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>9.619999999999999</v>
+        <v>-10.4</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>12.64</v>
+        <v>-1.36</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>1.52</v>
+        <v>-2.23</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>8.970000000000001</v>
+        <v>-4.39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.518</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13.54</v>
+        <v>39.07</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1095,43 +1085,41 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-17.28</v>
+        <v>-12.78</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-3.93</v>
+        <v>-1.86</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-0.59</v>
+        <v>-0.88</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>3.21</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.374</v>
+        <v>3.082</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>101.49</v>
+        <v>45.49</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1140,51 +1128,49 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="n">
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-9.99</v>
+        <v>3.07</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-0.66</v>
+        <v>0.3</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-1.02</v>
+        <v>-0.1</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-3.02</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.802</v>
+        <v>0.333</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>39.07</v>
+        <v>106.94</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1193,10 +1179,12 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -1208,34 +1196,34 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-13.01</v>
+        <v>-10.46</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-3.06</v>
+        <v>-1.07</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-0.51</v>
+        <v>-1.25</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>5.06</v>
+        <v>-2.27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.101</v>
+        <v>1.18</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45.49</v>
+        <v>33.19</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1245,50 +1233,52 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>2.96</v>
+        <v>-1.41</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>0.38</v>
+        <v>-5.59</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>0.15</v>
+        <v>3.52</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.337</v>
+        <v>0.418</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>106.94</v>
+        <v>102.25</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1297,53 +1287,53 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-10.7</v>
+        <v>-46.12</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-0.53</v>
+        <v>-15.65</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-0.45</v>
+        <v>0.18</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>0.29</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.18</v>
+        <v>1.128</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>33.19</v>
+        <v>47.73</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1353,52 +1343,48 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-2.31</v>
+        <v>-8.68</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-6.14</v>
+        <v>-6.83</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.78</v>
+        <v>-3.84</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>5.47</v>
+        <v>-4.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.426</v>
+        <v>0.853</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>102.25</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1410,52 +1396,46 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S16" s="2" t="n">
+      <c r="R16" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-46.19</v>
+        <v>-0.23</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-14.67</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>0.86</v>
+        <v>1.87</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>1.16</v>
+        <v>10.04</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.135</v>
+        <v>1.01</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>47.73</v>
+        <v>84.78</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1475,42 +1455,38 @@
       <c r="R17" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S17" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T17" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-8.5</v>
+        <v>-59.47</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-6.79</v>
+        <v>-22.55</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-3.71</v>
+        <v>-1.21</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-3.93</v>
+        <v>-3.34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.842</v>
+        <v>1.85</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>97.68000000000001</v>
+        <v>49.76</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1522,48 +1498,46 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-0.68</v>
+        <v>-22</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>7.07</v>
+        <v>-3.96</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.7</v>
+        <v>-0.37</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>9.06</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.029</v>
+        <v>2.219</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>84.78</v>
+        <v>61.93</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1573,9 +1547,11 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -1584,37 +1560,39 @@
         <v>-1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-60.02</v>
+        <v>18.27</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-21.64</v>
+        <v>15.88</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-1.39</v>
+        <v>0.74</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-3.29</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.846</v>
+        <v>1.044</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>49.76</v>
+        <v>27.11</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1626,50 +1604,46 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S20" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-23.05</v>
+        <v>50.94</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-4.79</v>
+        <v>20.74</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-0.17</v>
+        <v>3.55</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>5.85</v>
+        <v>-2.52</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.234</v>
+        <v>1.319</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>61.93</v>
+        <v>117.45</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1679,50 +1653,50 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>17.43</v>
+        <v>13.75</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>16.16</v>
+        <v>15.75</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.86</v>
+        <v>1.37</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>1.64</v>
+        <v>8.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.542</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>39.7</v>
+        <v>35.77</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1734,48 +1708,48 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>预1</t>
+          <t>预-1</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-24.31</v>
+        <v>-30.37</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-13.21</v>
+        <v>-15.95</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-1.4</v>
+        <v>-0.09</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-5.86</v>
+        <v>-3.52</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.052</v>
+        <v>0.671</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>27.11</v>
+        <v>19.95</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1787,48 +1761,46 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>48.96</v>
+        <v>48.95</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>21.26</v>
+        <v>17.66</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>3.13</v>
+        <v>3.38</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-1.95</v>
+        <v>-1.32</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.341</v>
+        <v>2.347</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>117.45</v>
+        <v>35.32</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1839,51 +1811,49 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R24" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>13.08</v>
+        <v>-30.58</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>17.14</v>
+        <v>-15.61</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>2.31</v>
+        <v>-0.9</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>9.77</v>
+        <v>-6.06</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.926</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>35.77</v>
+        <v>9.44</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1901,40 +1871,42 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-31.62</v>
+        <v>-3.66</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-15.47</v>
+        <v>-7.63</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>0.21</v>
+        <v>-2.51</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-4.47</v>
+        <v>-4.16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.677</v>
+        <v>3.358</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>19.95</v>
+        <v>12.25</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1946,46 +1918,44 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R26" s="2" t="inlineStr"/>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>47.02</v>
+        <v>9.25</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>18.31</v>
+        <v>1.15</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>3.34</v>
+        <v>0.58</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-0.1</v>
+        <v>-6.66</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.362</v>
+        <v>4.617</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>35.32</v>
+        <v>26.51</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1995,50 +1965,46 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-30.32</v>
+        <v>-0.33</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-15.46</v>
+        <v>1.2</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.62</v>
+        <v>-0.03</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-6.57</v>
+        <v>-0.04</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.521</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>9.44</v>
+        <v>13.54</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2050,48 +2016,44 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-3.55</v>
+        <v>-16.57</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-6.58</v>
+        <v>-2.77</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-0.82</v>
+        <v>-0.36</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-4.19</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.756</v>
+        <v>1.036</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>101.36</v>
+        <v>-0.84</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2113,34 +2075,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>42.77</v>
+        <v>33.13</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>25.52</v>
+        <v>10.77</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>3.73</v>
+        <v>-3.84</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>20.54</v>
+        <v>-12.21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.043</v>
+        <v>1.52</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-0.84</v>
+        <v>39.7</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2162,16 +2124,16 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>33.12</v>
+        <v>-26.09</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>11.05</v>
+        <v>-14.01</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-4.6</v>
+        <v>-3.04</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-13.5</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="31">
@@ -2186,7 +2148,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.671</v>
+        <v>1.659</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>-3.85</v>
@@ -2201,7 +2163,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2211,16 +2173,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>18.06</v>
+        <v>18.24</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>6.08</v>
+        <v>5.8</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-3.41</v>
+        <v>-3.14</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-10.08</v>
+        <v>-9.529999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2251,7 +2213,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-09 | 30 只</t>
+          <t>截至: 2026-09-10 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-09-11
</commit_message>
<xml_diff>
--- a/ETF_Swing_Pattern.xlsx
+++ b/ETF_Swing_Pattern.xlsx
@@ -628,19 +628,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>159920 SZ</t>
+          <t>159915 SZ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>恒生ETF</t>
+          <t>创业板ETF</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.466</v>
+        <v>3.341</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>99.02</v>
+        <v>12.25</v>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
@@ -652,46 +652,50 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="n">
-        <v>-1</v>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>-13.69</v>
+        <v>9.98</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-2.47</v>
+        <v>1.43</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-0.68</v>
+        <v>1.59</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>1.74</v>
+        <v>-7.43</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159920 SZ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>恒生ETF</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.667</v>
+        <v>1.457</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>95.98999999999999</v>
+        <v>99.02</v>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -703,7 +707,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -711,42 +715,38 @@
       <c r="R3" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-29.43</v>
+        <v>-13.72</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-9.32</v>
+        <v>-2.26</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.88</v>
+        <v>-2.49</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>2.24</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.769</v>
+        <v>0.658</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>101.36</v>
+        <v>90.17</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -756,62 +756,68 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>44.95</v>
+        <v>-30.18</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>26.98</v>
+        <v>-9.69</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>7.05</v>
+        <v>-2.65</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>20.88</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.821</v>
+        <v>1.759</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>101.36</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N5" s="2" t="n">
         <v>1</v>
       </c>
@@ -825,34 +831,34 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>-9.82</v>
+        <v>46.64</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>-1.7</v>
+        <v>27.17</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>-3.16</v>
+        <v>6.64</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>-8.720000000000001</v>
+        <v>19.84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.016</v>
+        <v>0.803</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44.27</v>
+        <v>4.26</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -864,46 +870,46 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="n">
+      <c r="R6" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-3.58</v>
+        <v>-11.04</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.61</v>
+        <v>-2.98</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.36</v>
+        <v>-3.89</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.17</v>
+        <v>-8.76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.742</v>
+        <v>2.981</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>33.48</v>
+        <v>55.83</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -913,9 +919,7 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
         <v>2</v>
       </c>
@@ -923,113 +927,115 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>9.140000000000001</v>
+        <v>-3.81</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>2.17</v>
+        <v>1.3</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.6</v>
+        <v>-0.99</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-1.4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.473</v>
+        <v>7.611</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>114.34</v>
+        <v>33.48</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>10.13</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>12.39</v>
+        <v>1.28</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>1.14</v>
+        <v>-0.16</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>9.039999999999999</v>
+        <v>-2.43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.369</v>
+        <v>3.419</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>101.49</v>
+        <v>114.34</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="n">
         <v>-9</v>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1041,34 +1047,34 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-10.4</v>
+        <v>10.47</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-1.36</v>
+        <v>11.53</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-2.23</v>
+        <v>0.13</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-4.39</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.506</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>39.07</v>
+        <v>6.73</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1080,46 +1086,46 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="n">
+      <c r="S10" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-12.78</v>
+        <v>-17.06</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-1.86</v>
+        <v>-4.68</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-0.88</v>
+        <v>-2.82</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>5.53</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3.082</v>
+        <v>0.365</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>45.49</v>
+        <v>89.56999999999999</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1128,49 +1134,51 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="n">
+      <c r="R11" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>3.07</v>
+        <v>-11.1</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.3</v>
+        <v>-1.57</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-0.1</v>
+        <v>-2.88</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.98</v>
+        <v>-3.06</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.333</v>
+        <v>0.788</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>106.94</v>
+        <v>79.75</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1179,51 +1187,51 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="n">
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-10.46</v>
+        <v>-13.46</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-1.07</v>
+        <v>-3.27</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-1.25</v>
+        <v>-3.07</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>-2.27</v>
+        <v>5.48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1.18</v>
+        <v>3.014</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>33.19</v>
+        <v>40.26</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1233,52 +1241,48 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-1.41</v>
+        <v>3.09</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-5.59</v>
+        <v>-1.05</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>3.52</v>
+        <v>-0.16</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>6.07</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.418</v>
+        <v>0.327</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>102.25</v>
+        <v>98.59</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1287,53 +1291,51 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S14" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-46.12</v>
+        <v>-10.76</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-15.65</v>
+        <v>-1.99</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>0.18</v>
+        <v>-2.35</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>-1.01</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.128</v>
+        <v>1.167</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>47.73</v>
+        <v>33.19</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1343,48 +1345,52 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="n">
+      <c r="R15" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V15" s="2" t="n">
-        <v>-8.68</v>
+        <v>-0.86</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-6.83</v>
+        <v>-5.8</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-3.84</v>
+        <v>2.53</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>-4.54</v>
+        <v>5.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.853</v>
+        <v>0.412</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>97.68000000000001</v>
+        <v>80.06</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1396,46 +1402,50 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-0.23</v>
+        <v>-46.94</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>9.050000000000001</v>
+        <v>-16.02</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1.87</v>
+        <v>-2.96</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>10.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.01</v>
+        <v>1.022</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>84.78</v>
+        <v>-3.59</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1447,46 +1457,48 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="n">
-        <v>-1</v>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-59.47</v>
+        <v>33.03</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-22.55</v>
+        <v>10.09</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-1.21</v>
+        <v>-1.25</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-3.34</v>
+        <v>-13.25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.85</v>
+        <v>0.847</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>49.76</v>
+        <v>99.92</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1498,46 +1510,48 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr"/>
-      <c r="S18" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-22</v>
+        <v>0.03</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-3.96</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.37</v>
+        <v>0.86</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>5.68</v>
+        <v>10.89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.219</v>
+        <v>1.015</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>61.93</v>
+        <v>11.5</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1548,51 +1562,49 @@
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="n">
-        <v>-13</v>
+        <v>9</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>18.27</v>
+        <v>-59.03</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>15.88</v>
+        <v>-21.39</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.74</v>
+        <v>-1.85</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>0.78</v>
+        <v>-0.75</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.044</v>
+        <v>2.201</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>27.11</v>
+        <v>85.05</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1602,48 +1614,50 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N20" s="2" t="n">
         <v>3</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>50.94</v>
+        <v>19.48</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>20.74</v>
+        <v>15.8</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>3.55</v>
+        <v>-0.72</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>-2.52</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.319</v>
+        <v>1.487</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>117.45</v>
+        <v>12.11</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1653,9 +1667,11 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -1669,34 +1685,34 @@
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>13.75</v>
+        <v>-27.34</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>15.75</v>
+        <v>-15.17</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>1.37</v>
+        <v>-3.15</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>8.48</v>
+        <v>-7.74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8080000000000001</v>
+        <v>1.047</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>35.77</v>
+        <v>24.85</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1708,48 +1724,46 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-30.37</v>
+        <v>52.97</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-15.95</v>
+        <v>21.88</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.09</v>
+        <v>6.79</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>-3.52</v>
+        <v>-4.43</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.671</v>
+        <v>0.793</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>19.95</v>
+        <v>35.77</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1761,46 +1775,46 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>48.95</v>
+        <v>-28.81</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>17.66</v>
+        <v>-16.79</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>3.38</v>
+        <v>-0.51</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-1.32</v>
+        <v>-4.52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2.347</v>
+        <v>0.675</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>35.32</v>
+        <v>26.58</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1810,50 +1824,48 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="n">
-        <v>9</v>
-      </c>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
-      <c r="T24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-30.58</v>
+        <v>50.81</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-15.61</v>
+        <v>19.16</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.9</v>
+        <v>6.22</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-6.06</v>
+        <v>-3.75</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.926</v>
+        <v>2.302</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>9.44</v>
+        <v>10.28</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1863,50 +1875,50 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N25" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S25" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-3.66</v>
+        <v>-30.45</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-7.63</v>
+        <v>-16.42</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-2.51</v>
+        <v>-0.98</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-4.16</v>
+        <v>-7.15</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>159915 SZ</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>创业板ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>3.358</v>
+        <v>0.91</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>12.25</v>
+        <v>3.17</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1918,44 +1930,46 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>9.25</v>
+        <v>-3.91</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>1.15</v>
+        <v>-8.41</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>0.58</v>
+        <v>-1.83</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-6.66</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>4.617</v>
+        <v>1.639</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>26.51</v>
+        <v>-4.94</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1972,39 +1986,43 @@
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-0.33</v>
+        <v>18.24</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>1.2</v>
+        <v>5.36</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-0.03</v>
+        <v>-1.34</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>-0.04</v>
+        <v>-9.890000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.521</v>
+        <v>4.579</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>13.54</v>
+        <v>10.81</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2016,7 +2034,7 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -2026,34 +2044,34 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>-16.57</v>
+        <v>-0.11</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-2.77</v>
+        <v>1.21</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-0.36</v>
+        <v>-0.01</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>3.38</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1.036</v>
+        <v>1.111</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-0.84</v>
+        <v>5.68</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2065,7 +2083,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2075,34 +2093,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>33.13</v>
+        <v>-9.460000000000001</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>10.77</v>
+        <v>-7.41</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-3.84</v>
+        <v>-2.98</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-12.21</v>
+        <v>-5.38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.52</v>
+        <v>1.814</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>39.7</v>
+        <v>93.77</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2124,34 +2142,34 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-26.09</v>
+        <v>-22</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-14.01</v>
+        <v>-4.93</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-3.04</v>
+        <v>-3.42</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-6.1</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.659</v>
+        <v>1.292</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-3.85</v>
+        <v>117.45</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2163,7 +2181,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2173,16 +2191,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>18.24</v>
+        <v>14.43</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>5.8</v>
+        <v>14.24</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-3.14</v>
+        <v>-0.03</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-9.529999999999999</v>
+        <v>5.32</v>
       </c>
     </row>
   </sheetData>
@@ -2213,7 +2231,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-10 | 30 只</t>
+          <t>截至: 2026-09-11 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>